<commit_message>
Initial commit for SCR automation project
</commit_message>
<xml_diff>
--- a/reference/Duties Per Unit.xlsx
+++ b/reference/Duties Per Unit.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prajw\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prajw\OneDrive\Documents\Projects\scr_automation\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD2A7B88-7969-40D8-B6AF-1069B3C6955D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4726ACC-1D1C-4114-B19F-BEA2BD95474F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11235" xr2:uid="{55EB7257-F8C4-436D-8C05-255F0E4A01B2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{55EB7257-F8C4-436D-8C05-255F0E4A01B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -113,9 +113,6 @@
     <t>CPCCCA3008 - Construct eaves</t>
   </si>
   <si>
-    <t>Construct leaves</t>
-  </si>
-  <si>
     <t>CPCCCA3010 - Install windows and doors</t>
   </si>
   <si>
@@ -351,6 +348,9 @@
   </si>
   <si>
     <t>Serial No</t>
+  </si>
+  <si>
+    <t>Construct eaves</t>
   </si>
 </sst>
 </file>
@@ -777,7 +777,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -788,7 +788,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>2</v>
@@ -799,7 +799,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>4</v>
@@ -810,7 +810,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>8</v>
@@ -832,7 +832,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>10</v>
@@ -843,7 +843,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>12</v>
@@ -854,7 +854,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>14</v>
@@ -865,7 +865,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>16</v>
@@ -876,7 +876,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>18</v>
@@ -887,7 +887,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>20</v>
@@ -898,7 +898,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>22</v>
@@ -909,255 +909,255 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>